<commit_message>
feat(checkout): thanh toán online FoxPay/NAPAS + sheet Common 4 cột dịch vụ
Automation:
- ckcommon.shared TC_CKCOMMON.61: hoàn tất thanh toán thẻ nội địa qua cổng FoxPay/NAPAS
- pages/common/foxpay-gateway.page.ts: page object cổng FoxPay (form thẻ → OTP → success)
- camera-checkout-common.spec.ts: Camera chạy CKCOMMON (prefix [Camera])
- checkout.data.ts: sửa data thẻ ATM (issueDate 03/07 + otp) — fix case online trước đây fail
  do Excel convert "03/07" thành "2026-03-07" → cổng báo sai ngày hết hạn

Report/sync:
- sheet Checkout_Common: 4 block cố định Internet/Camera/AP/SmartTV (sync_tc_checkout.py)
- sync-tc-results.md: tài liệu hóa quy ước ghi nhận per-dịch-vụ

Kèm: camera page/spec, cập nhật tài liệu + data test Voucher.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ecom-pdh/03_test-cases/functional/chucnang_Voucher/AI_ISC_ecom-pdh_v1.1_TC_voucher_ui_v1.0.xlsx
+++ b/ecom-pdh/03_test-cases/functional/chucnang_Voucher/AI_ISC_ecom-pdh_v1.1_TC_voucher_ui_v1.0.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12390" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Voucher_UI_Checkout" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Voucher_UI_Checkout" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="162913" fullCalcOnLoad="1"/>
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -84,8 +84,11 @@
       <name val="Calibri"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -120,6 +123,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE699"/>
       </patternFill>
     </fill>
   </fills>
@@ -390,7 +398,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -483,6 +491,14 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -850,16 +866,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:N33"/>
+  <dimension ref="A3:N45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="2" min="1" max="1"/>
     <col width="15" customWidth="1" style="2" min="2" max="2"/>
     <col width="12" customWidth="1" style="2" min="3" max="3"/>
-    <col width="55" customWidth="1" style="2" min="4" max="4"/>
-    <col width="44" customWidth="1" style="2" min="5" max="5"/>
-    <col width="52" customWidth="1" style="2" min="6" max="6"/>
-    <col width="58" customWidth="1" style="2" min="7" max="7"/>
+    <col width="45" customWidth="1" style="2" min="4" max="4"/>
+    <col width="38" customWidth="1" style="2" min="5" max="5"/>
+    <col width="42" customWidth="1" style="2" min="6" max="6"/>
+    <col width="55" customWidth="1" style="2" min="7" max="7"/>
     <col width="14" customWidth="1" style="2" min="8" max="8"/>
     <col width="15" customWidth="1" style="2" min="9" max="9"/>
     <col width="12" customWidth="1" style="2" min="10" max="10"/>
@@ -2009,7 +2025,7 @@
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>TC_VOU.18</t>
+          <t>TC_VOU.19</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
@@ -2049,8 +2065,598 @@
       <c r="M33" s="8" t="n"/>
       <c r="N33" s="8" t="n"/>
     </row>
+    <row r="34" ht="18" customHeight="1" s="2">
+      <c r="A34" s="42" t="n"/>
+      <c r="B34" s="43" t="inlineStr">
+        <is>
+          <t>Nhóm 7: Giao diện Modal Chọn ưu đãi — Figma UI Analysis (DOC-VOUCHER-UI-01)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="80" customHeight="1" s="2">
+      <c r="A35" s="44" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B35" s="44" t="inlineStr">
+        <is>
+          <t>TC_VOU.20</t>
+        </is>
+      </c>
+      <c r="C35" s="44" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D35" s="44" t="inlineStr">
+        <is>
+          <t>Kiểm tra hiển thị section "Chọn ưu đãi" mặc định trên trang Cart (chưa áp voucher)</t>
+        </is>
+      </c>
+      <c r="E35" s="44" t="inlineStr">
+        <is>
+          <t>- KH đang ở trang Giỏ hàng (Cart)
+- Chưa áp dụng voucher nào
+- Có ít nhất 1 sản phẩm trong giỏ</t>
+        </is>
+      </c>
+      <c r="F35" s="44" t="inlineStr">
+        <is>
+          <t>1. Truy cập trang Cart
+2. Quan sát khu vực Thông tin thanh toán (cột phải)
+3. Tìm phần nhập mã ưu đãi</t>
+        </is>
+      </c>
+      <c r="G35" s="44" t="inlineStr">
+        <is>
+          <t>- Link "Nhập các mã ưu đãi của bạn" hiển thị bên dưới dòng tạm tính
+- Không có tên voucher hay số tiền giảm nào được hiển thị
+- Nút "Tiếp tục" vẫn active</t>
+        </is>
+      </c>
+      <c r="H35" s="44" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I35" s="44" t="n"/>
+      <c r="J35" s="44" t="n"/>
+      <c r="K35" s="44" t="n"/>
+      <c r="L35" s="44" t="n"/>
+    </row>
+    <row r="36" ht="80" customHeight="1" s="2">
+      <c r="A36" s="44" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B36" s="44" t="inlineStr">
+        <is>
+          <t>TC_VOU.21</t>
+        </is>
+      </c>
+      <c r="C36" s="44" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D36" s="44" t="inlineStr">
+        <is>
+          <t>Kiểm tra hiển thị section "Chọn ưu đãi" mặc định trên trang Checkout đầy đủ (chưa áp voucher)</t>
+        </is>
+      </c>
+      <c r="E36" s="44" t="inlineStr">
+        <is>
+          <t>- KH đang ở trang Checkout đầy đủ (bước Thanh toán)
+- Chưa áp dụng voucher nào
+- Đã điền thông tin cá nhân và chọn PTTT</t>
+        </is>
+      </c>
+      <c r="F36" s="44" t="inlineStr">
+        <is>
+          <t>1. Truy cập trang Checkout đầy đủ
+2. Quan sát section "Thông tin thanh toán" (cột phải)
+3. Ghi nhận trạng thái khu vực voucher</t>
+        </is>
+      </c>
+      <c r="G36" s="44" t="inlineStr">
+        <is>
+          <t>- Button/link "Chọn ưu đãi" hiển thị trong section Thông tin thanh toán
+- Button "Áp dụng" ở trạng thái disabled hoặc là link dạng text
+- Không có tên voucher hay số tiền giảm nào được hiển thị
+- Dòng "Cần thanh toán" = giá gốc chưa có discount</t>
+        </is>
+      </c>
+      <c r="H36" s="44" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I36" s="44" t="n"/>
+      <c r="J36" s="44" t="n"/>
+      <c r="K36" s="44" t="n"/>
+      <c r="L36" s="44" t="n"/>
+    </row>
+    <row r="37" ht="80" customHeight="1" s="2">
+      <c r="A37" s="44" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B37" s="44" t="inlineStr">
+        <is>
+          <t>TC_VOU.22</t>
+        </is>
+      </c>
+      <c r="C37" s="44" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D37" s="44" t="inlineStr">
+        <is>
+          <t>Kiểm tra cấu trúc 2 tab trong Modal "Chọn ưu đãi" (tab Mã giảm giá / Ưu đãi)</t>
+        </is>
+      </c>
+      <c r="E37" s="44" t="inlineStr">
+        <is>
+          <t>- KH đang ở trang Cart hoặc Checkout
+- Hệ thống có ít nhất 1 voucher khả dụng cho tài khoản/đơn hàng
+- Đã chọn PTTT</t>
+        </is>
+      </c>
+      <c r="F37" s="44" t="inlineStr">
+        <is>
+          <t>1. Click link "Nhập các mã ưu đãi của bạn" hoặc button "Chọn ưu đãi"
+2. Quan sát cấu trúc tổng thể modal
+3. Click tab "Mã giảm giá"
+4. Ghi nhận danh sách voucher hiển thị
+5. Click tab "Ưu đãi"
+6. Ghi nhận danh sách voucher thay đổi</t>
+        </is>
+      </c>
+      <c r="G37" s="44" t="inlineStr">
+        <is>
+          <t>- Modal hiển thị: title "Chọn ưu đãi", nút X ở góc trên phải
+- 2 tab hiển thị: "Mã giảm giá" và "Ưu đãi"; tab được click sẽ được highlight (active state)
+- Nội dung voucher trong mỗi tab hiển thị đúng theo phân loại
+- Button "Xác nhận" / "Đồng ý" hiển thị ở cuối modal</t>
+        </is>
+      </c>
+      <c r="H37" s="44" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I37" s="44" t="n"/>
+      <c r="J37" s="44" t="n"/>
+      <c r="K37" s="44" t="n"/>
+      <c r="L37" s="44" t="n"/>
+    </row>
+    <row r="38" ht="80" customHeight="1" s="2">
+      <c r="A38" s="44" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B38" s="44" t="inlineStr">
+        <is>
+          <t>TC_VOU.23</t>
+        </is>
+      </c>
+      <c r="C38" s="44" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D38" s="44" t="inlineStr">
+        <is>
+          <t>Kiểm tra các thành phần hiển thị trong Voucher Card Item</t>
+        </is>
+      </c>
+      <c r="E38" s="44" t="inlineStr">
+        <is>
+          <t>- Modal "Chọn ưu đãi" đang mở
+- Có ít nhất 1 voucher card trong danh sách</t>
+        </is>
+      </c>
+      <c r="F38" s="44" t="inlineStr">
+        <is>
+          <t>1. Quan sát chi tiết 1 voucher card trong danh sách
+2. Kiểm tra từng thành phần trên card
+3. Ghi nhận link "Điều kiện" có hiển thị không</t>
+        </is>
+      </c>
+      <c r="G38" s="44" t="inlineStr">
+        <is>
+          <t>Mỗi voucher card hiển thị đầy đủ:
+(1) Icon/thumbnail màu đặc trưng (cam/xanh)
+(2) Tên voucher in đậm (VD: "Giảm 10%, tối đa 100k")
+(3) Mô tả ngắn (VD: "Áp dụng thanh toán các đơn hàng CDD")
+(4) Ngày hết hạn (VD: 30.08.2025)
+(5) Control chọn (radio hoặc checkbox)
+(6) Link "Điều kiện" điều hướng đến màn chi tiết</t>
+        </is>
+      </c>
+      <c r="H38" s="44" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I38" s="44" t="n"/>
+      <c r="J38" s="44" t="n"/>
+      <c r="K38" s="44" t="n"/>
+      <c r="L38" s="44" t="n"/>
+    </row>
+    <row r="39" ht="80" customHeight="1" s="2">
+      <c r="A39" s="44" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B39" s="44" t="inlineStr">
+        <is>
+          <t>TC_VOU.24</t>
+        </is>
+      </c>
+      <c r="C39" s="44" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D39" s="44" t="inlineStr">
+        <is>
+          <t>Kiểm tra Modal Empty State khi không có voucher khả dụng cho đơn hàng</t>
+        </is>
+      </c>
+      <c r="E39" s="44" t="inlineStr">
+        <is>
+          <t>- KH đang ở trang Cart hoặc Checkout
+- Tài khoản/đơn hàng không có voucher khả dụng nào (API trả list rỗng)
+- Đã chọn PTTT</t>
+        </is>
+      </c>
+      <c r="F39" s="44" t="inlineStr">
+        <is>
+          <t>1. Click link/button "Chọn ưu đãi"
+2. Chờ modal mở
+3. Quan sát nội dung bên trong modal</t>
+        </is>
+      </c>
+      <c r="G39" s="44" t="inlineStr">
+        <is>
+          <t>- Modal mở, hiển thị title "Chọn ưu đãi" và nút X
+- Không có danh sách voucher nào
+- Hiển thị hình minh hoạ empty state
+- Text thông báo: "Tất tiếc, ngay lúc này chưa có ưu đãi."
+- Không hiển thị button "Xác nhận"</t>
+        </is>
+      </c>
+      <c r="H39" s="44" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I39" s="44" t="n"/>
+      <c r="J39" s="44" t="n"/>
+      <c r="K39" s="44" t="n"/>
+      <c r="L39" s="44" t="n"/>
+    </row>
+    <row r="40" ht="80" customHeight="1" s="2">
+      <c r="A40" s="44" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B40" s="44" t="inlineStr">
+        <is>
+          <t>TC_VOU.25</t>
+        </is>
+      </c>
+      <c r="C40" s="44" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D40" s="44" t="inlineStr">
+        <is>
+          <t>Kiểm tra màn hình Chi tiết Ưu đãi hiển thị đầy đủ thông tin và section Điều khoản</t>
+        </is>
+      </c>
+      <c r="E40" s="44" t="inlineStr">
+        <is>
+          <t>- Modal "Chọn ưu đãi" đang mở
+- Có ít nhất 1 voucher card trong danh sách có link "Điều kiện"</t>
+        </is>
+      </c>
+      <c r="F40" s="44" t="inlineStr">
+        <is>
+          <t>1. Click link "Điều kiện" trên 1 voucher card
+2. Quan sát màn hình Chi tiết Ưu đãi
+3. Click vào section "Xem chi tiết" / "Điều khoản" để expand
+4. Đọc nội dung bullet list điều khoản</t>
+        </is>
+      </c>
+      <c r="G40" s="44" t="inlineStr">
+        <is>
+          <t>Màn hình Chi tiết Ưu đãi hiển thị đầy đủ:
+(1) Header banner: icon + tên voucher + mô tả + HSD
+(2) Hạn sử dụng (từ ngày → đến ngày, định dạng dd/MM/yyyy)
+(3) Mô tả Ưu đãi (VD: "Giảm 10%... tối đa 100.000đ, đơn tối thiểu 500k")
+(4) Áp dụng cho dịch vụ (VD: "Tất cả sản phẩm dịch vụ")
+(5) Phương thức Thanh toán (VD: "Thanh toán tại nhà (COD)")
+(6) Section "Xem chi tiết" expandable → hiển thị bullet list điều khoản
+(7) Button "Sử dụng ưu đãi" ở cuối màn hình</t>
+        </is>
+      </c>
+      <c r="H40" s="44" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I40" s="44" t="n"/>
+      <c r="J40" s="44" t="n"/>
+      <c r="K40" s="44" t="n"/>
+      <c r="L40" s="44" t="n"/>
+    </row>
+    <row r="41" ht="80" customHeight="1" s="2">
+      <c r="A41" s="44" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B41" s="44" t="inlineStr">
+        <is>
+          <t>TC_VOU.26</t>
+        </is>
+      </c>
+      <c r="C41" s="44" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D41" s="44" t="inlineStr">
+        <is>
+          <t>Kiểm tra button "Sử dụng ưu đãi" từ màn hình Chi tiết áp dụng voucher và quay về Checkout</t>
+        </is>
+      </c>
+      <c r="E41" s="44" t="inlineStr">
+        <is>
+          <t>- KH đang xem màn hình Chi tiết Ưu đãi của voucher V (VD: giảm 10%, tối đa 100k)
+- Voucher V còn hợp lệ
+- KH chưa áp dụng voucher nào</t>
+        </is>
+      </c>
+      <c r="F41" s="44" t="inlineStr">
+        <is>
+          <t>1. Ghi nhận tên và giá trị giảm của voucher V
+2. Click button "Sử dụng ưu đãi" ở cuối màn hình
+3. Quan sát màn hình sau khi click</t>
+        </is>
+      </c>
+      <c r="G41" s="44" t="inlineStr">
+        <is>
+          <t>- Màn hình Chi tiết đóng
+- KH được điều hướng lại trang Checkout
+- Tên/mã voucher V hiển thị trong section "Thông tin thanh toán"
+- Số tiền giảm và "Cần thanh toán" cập nhật đúng theo giá trị voucher V</t>
+        </is>
+      </c>
+      <c r="H41" s="44" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I41" s="44" t="n"/>
+      <c r="J41" s="44" t="n"/>
+      <c r="K41" s="44" t="n"/>
+      <c r="L41" s="44" t="n"/>
+    </row>
+    <row r="42" ht="80" customHeight="1" s="2">
+      <c r="A42" s="44" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B42" s="44" t="inlineStr">
+        <is>
+          <t>TC_VOU.27</t>
+        </is>
+      </c>
+      <c r="C42" s="44" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D42" s="44" t="inlineStr">
+        <is>
+          <t>Kiểm tra voucher đã áp dụng hiển thị trên sticky bottom bar khi dùng Mobile</t>
+        </is>
+      </c>
+      <c r="E42" s="44" t="inlineStr">
+        <is>
+          <t>- KH sử dụng thiết bị Mobile (iOS/Android, viewport ≤768px)
+- KH đang ở trang Checkout mobile
+- Đã áp dụng voucher V thành công (VD: Giảm 200k)</t>
+        </is>
+      </c>
+      <c r="F42" s="44" t="inlineStr">
+        <is>
+          <t>1. Truy cập trang Checkout trên thiết bị mobile
+2. Áp dụng voucher V hợp lệ
+3. Quan sát sticky bottom bar ở phía dưới màn hình
+4. Ghi nhận thông tin hiển thị trong bar</t>
+        </is>
+      </c>
+      <c r="G42" s="44" t="inlineStr">
+        <is>
+          <t>- Sticky bottom bar hiển thị: tên/mã voucher V (hoặc icon voucher)
+- Tổng "Cần thanh toán" trong sticky bar đã cập nhật sau giảm (= giá gốc − giá trị voucher)
+- Button "Tiếp tục" vẫn active và có thể click</t>
+        </is>
+      </c>
+      <c r="H42" s="44" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I42" s="44" t="n"/>
+      <c r="J42" s="44" t="n"/>
+      <c r="K42" s="44" t="n"/>
+      <c r="L42" s="44" t="n"/>
+    </row>
+    <row r="43" ht="80" customHeight="1" s="2">
+      <c r="A43" s="45" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B43" s="45" t="inlineStr">
+        <is>
+          <t>TC_VOU.28</t>
+        </is>
+      </c>
+      <c r="C43" s="45" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D43" s="45" t="inlineStr">
+        <is>
+          <t>Kiểm tra hệ thống lọc voucher theo điều kiện đơn hàng trong Modal Chọn ưu đãi</t>
+        </is>
+      </c>
+      <c r="E43" s="45" t="inlineStr">
+        <is>
+          <t>- KH mở Modal "Chọn ưu đãi"
+- Hệ thống có voucher nhưng một số không match điều kiện PTTT/dịch vụ của đơn hàng</t>
+        </is>
+      </c>
+      <c r="F43" s="45" t="inlineStr">
+        <is>
+          <t>1. Chọn PTTT cụ thể (VD: Momo)
+2. Click "Chọn ưu đãi"
+3. Quan sát danh sách voucher trong modal</t>
+        </is>
+      </c>
+      <c r="G43" s="45" t="inlineStr">
+        <is>
+          <t>[BLOCKED – CLA-FIGMA-001: cần BA xác nhận quy tắc filter — điều kiện nào để voucher appear/hidden trong list (theo PTTT, theo dịch vụ, theo KH...)?]</t>
+        </is>
+      </c>
+      <c r="H43" s="45" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I43" s="45" t="n"/>
+      <c r="J43" s="45" t="n"/>
+      <c r="K43" s="45" t="n"/>
+      <c r="L43" s="45" t="n"/>
+    </row>
+    <row r="44" ht="80" customHeight="1" s="2">
+      <c r="A44" s="45" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B44" s="45" t="inlineStr">
+        <is>
+          <t>TC_VOU.29</t>
+        </is>
+      </c>
+      <c r="C44" s="45" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D44" s="45" t="inlineStr">
+        <is>
+          <t>Kiểm tra thông báo hệ thống khi PTTT không match điều kiện voucher đã áp dụng</t>
+        </is>
+      </c>
+      <c r="E44" s="45" t="inlineStr">
+        <is>
+          <t>- KH đã áp dụng voucher V có điều kiện PTTT = COD
+- KH đang ở trang Checkout, voucher V đang hiển thị</t>
+        </is>
+      </c>
+      <c r="F44" s="45" t="inlineStr">
+        <is>
+          <t>1. Ghi nhận voucher V đang được áp dụng (PTTT = COD)
+2. Thay đổi PTTT sang Momo
+3. Quan sát phản hồi của hệ thống</t>
+        </is>
+      </c>
+      <c r="G44" s="45" t="inlineStr">
+        <is>
+          <t>[BLOCKED – CLA-FIGMA-004: cần BA/Dev xác nhận luồng xử lý khi PTTT không match voucher — popup thông báo? snackbar? auto remove voucher? (Figma Note N4 của uConn_Nam chưa có answer)]</t>
+        </is>
+      </c>
+      <c r="H44" s="45" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I44" s="45" t="n"/>
+      <c r="J44" s="45" t="n"/>
+      <c r="K44" s="45" t="n"/>
+      <c r="L44" s="45" t="n"/>
+    </row>
+    <row r="45" ht="80" customHeight="1" s="2">
+      <c r="A45" s="45" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B45" s="45" t="inlineStr">
+        <is>
+          <t>TC_VOU.30</t>
+        </is>
+      </c>
+      <c r="C45" s="45" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D45" s="45" t="inlineStr">
+        <is>
+          <t>Kiểm tra hiển thị Voucher Card ở trạng thái disabled/đã dùng/hết hạn</t>
+        </is>
+      </c>
+      <c r="E45" s="45" t="inlineStr">
+        <is>
+          <t>- KH mở Modal "Chọn ưu đãi"
+- Danh sách có chứa voucher đã sử dụng hoặc hết hạn</t>
+        </is>
+      </c>
+      <c r="F45" s="45" t="inlineStr">
+        <is>
+          <t>1. Click "Chọn ưu đãi"
+2. Quan sát voucher card không khả dụng trong danh sách
+3. Click vào card không khả dụng
+4. Quan sát hành vi của card</t>
+        </is>
+      </c>
+      <c r="G45" s="45" t="inlineStr">
+        <is>
+          <t>[BLOCKED – CLA-FIGMA-002: cần Designer/BA xác nhận UI state — Figma (Case C8) chưa thiết kế state này. Cần confirm: dimmed? text 'Đã dùng'? strike-through? không cho click?]</t>
+        </is>
+      </c>
+      <c r="H45" s="45" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I45" s="45" t="n"/>
+      <c r="J45" s="45" t="n"/>
+      <c r="K45" s="45" t="n"/>
+      <c r="L45" s="45" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="15">
+    <mergeCell ref="B34:L34"/>
     <mergeCell ref="B9:K9"/>
     <mergeCell ref="B30:K30"/>
     <mergeCell ref="C7:C8"/>

</xml_diff>